<commit_message>
ENG-067: gtm docs and planning data on D-016 pricing: 49 EUR list, 39 EUR founding price only with its qualifier
Spoken scripts use the founder line, written channels name only 49 EUR and the founding
price „im persönlichen Gespräch“. Break-even maths at 49 EUR (café 6 EUR: 9 visits, bakery
3 EUR: 17, salon 45 EUR: 2). Funnel and month-one models count shops, not revenue: notes
changed, totals unchanged. Angle IDs kept; CORE-09 hook rewritten to 49 EUR.
</commit_message>
<xml_diff>
--- a/gtm/data/funnel-model.xlsx
+++ b/gtm/data/funnel-model.xlsx
@@ -79,7 +79,17 @@
       </c>
       <c r="G2" t="inlineStr">
         <is>
-          <t>Fixed goal. Price stays 39 EUR / location / month.</t>
+          <t>Fixed goal. List price 49 EUR / location / month; founding shops pay 39 EUR</t>
+        </is>
+      </c>
+      <c r="H2" t="inlineStr">
+        <is>
+          <t> fixed for their contract term (D-016). The model counts shops</t>
+        </is>
+      </c>
+      <c r="I2" t="inlineStr">
+        <is>
+          <t> not revenue.</t>
         </is>
       </c>
     </row>
@@ -1003,7 +1013,12 @@
       </c>
       <c r="J9" t="inlineStr">
         <is>
-          <t>Close = agrees to the €39 terms (paid start only after the owner clears the commercial gates).</t>
+          <t>Close = agrees to the written terms</t>
+        </is>
+      </c>
+      <c r="K9" t="inlineStr">
+        <is>
+          <t> 49 € list or 39 € founding price (paid start only after the owner clears the commercial gates).</t>
         </is>
       </c>
     </row>

</xml_diff>